<commit_message>
Update transaction Excel file with new data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8589FC-558D-49A9-B053-9E057D702821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2E7D78-865E-4102-9C11-BAFC462EEF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8301,7 +8301,7 @@
         <v>31</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>348</v>
+        <v>17</v>
       </c>
       <c r="D16" s="6">
         <v>15</v>

</xml_diff>

<commit_message>
Update all.xlsx with latest transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A447340E-66E0-4B74-A4F3-CD1B2BF3AB20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76032464-E053-4BC7-9329-7AE4BCCB2EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8376" uniqueCount="2343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8378" uniqueCount="2344">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7066,6 +7066,9 @@
   </si>
   <si>
     <t>SALINV-01-01-26250</t>
+  </si>
+  <si>
+    <t>4667</t>
   </si>
 </sst>
 </file>
@@ -12738,8 +12741,8 @@
         <f t="shared" si="2"/>
         <v>6900</v>
       </c>
-      <c r="G134" s="42">
-        <v>40667</v>
+      <c r="G134" s="42" t="s">
+        <v>2343</v>
       </c>
       <c r="H134" s="11" t="s">
         <v>152</v>
@@ -12774,8 +12777,8 @@
         <f t="shared" si="2"/>
         <v>1350</v>
       </c>
-      <c r="G135" s="42">
-        <v>40667</v>
+      <c r="G135" s="42" t="s">
+        <v>2343</v>
       </c>
       <c r="H135" s="11" t="s">
         <v>152</v>
@@ -62146,14 +62149,14 @@
         <v>17</v>
       </c>
       <c r="D1508" s="6">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E1508" s="6">
         <v>936</v>
       </c>
       <c r="F1508" s="63">
         <f t="shared" si="23"/>
-        <v>76752</v>
+        <v>26208</v>
       </c>
       <c r="G1508" s="42">
         <v>138</v>
@@ -64576,7 +64579,7 @@
     <row r="1576" spans="1:11" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="F1576" s="67">
         <f>SUM(F2:F1575)</f>
-        <v>31323125.786196016</v>
+        <v>31272581.786196016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update all.xlsx with the latest transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76032464-E053-4BC7-9329-7AE4BCCB2EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10065211-AC79-4B08-9724-B58FD3835F20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59107,14 +59107,14 @@
         <v>40</v>
       </c>
       <c r="D1423" s="6">
-        <v>52400</v>
+        <v>52.4</v>
       </c>
       <c r="E1423" s="6">
         <v>90</v>
       </c>
       <c r="F1423" s="63">
         <f t="shared" si="22"/>
-        <v>4716000</v>
+        <v>4716</v>
       </c>
       <c r="G1423" s="42">
         <v>13910</v>
@@ -64579,7 +64579,7 @@
     <row r="1576" spans="1:11" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="F1576" s="67">
         <f>SUM(F2:F1575)</f>
-        <v>31272581.786196016</v>
+        <v>26561297.786196016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update all.xlsx with revised transaction data
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590BD02C-2945-4DE5-892A-58A80FA2AC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56A6023-71DF-4007-9AE5-C1A077E83A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7083,9 +7083,6 @@
     <t>DH004497-26</t>
   </si>
   <si>
-    <t>RAW-M-2026-0001755</t>
-  </si>
-  <si>
     <t>ES001379-26</t>
   </si>
   <si>
@@ -7098,7 +7095,10 @@
     <t>6263</t>
   </si>
   <si>
-    <t>RAW-S-2026-000080</t>
+    <t>RAW/S/2026/000080</t>
+  </si>
+  <si>
+    <t>RAW/M/2026/0001755</t>
   </si>
 </sst>
 </file>
@@ -7955,7 +7955,7 @@
     <col min="4" max="4" width="12" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" style="66" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.85546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.28515625" style="49" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" style="60" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.42578125" style="49" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.28515625" style="49" bestFit="1" customWidth="1"/>
@@ -35361,7 +35361,7 @@
     <row r="762" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A762" s="25"/>
       <c r="B762" s="42" t="s">
-        <v>2350</v>
+        <v>2349</v>
       </c>
       <c r="C762" s="42" t="s">
         <v>17</v>
@@ -35377,7 +35377,7 @@
         <v>12631.6</v>
       </c>
       <c r="G762" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H762" s="11" t="s">
         <v>1284</v>
@@ -35395,7 +35395,7 @@
     <row r="763" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A763" s="25"/>
       <c r="B763" s="42" t="s">
-        <v>2351</v>
+        <v>2350</v>
       </c>
       <c r="C763" s="42" t="s">
         <v>17</v>
@@ -35411,7 +35411,7 @@
         <v>965</v>
       </c>
       <c r="G763" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H763" s="11">
         <v>46297</v>
@@ -35420,7 +35420,7 @@
         <v>1285</v>
       </c>
       <c r="J763" s="42" t="s">
-        <v>2352</v>
+        <v>2351</v>
       </c>
       <c r="K763" s="11" t="s">
         <v>1286</v>
@@ -35447,7 +35447,7 @@
         <v>41650</v>
       </c>
       <c r="G764" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H764" s="11" t="s">
         <v>1284</v>
@@ -35483,7 +35483,7 @@
         <v>960</v>
       </c>
       <c r="G765" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H765" s="11" t="s">
         <v>1284</v>
@@ -35519,7 +35519,7 @@
         <v>49980</v>
       </c>
       <c r="G766" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H766" s="11" t="s">
         <v>1284</v>
@@ -35555,7 +35555,7 @@
         <v>58100</v>
       </c>
       <c r="G767" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H767" s="11" t="s">
         <v>1284</v>
@@ -35591,7 +35591,7 @@
         <v>14450</v>
       </c>
       <c r="G768" s="42" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="H768" s="11" t="s">
         <v>1284</v>
@@ -42630,11 +42630,11 @@
         <v>5</v>
       </c>
       <c r="E964" s="6">
-        <v>26116.6</v>
+        <v>2476</v>
       </c>
       <c r="F964" s="63">
         <f t="shared" ref="F964:F1027" si="15">E964*D964</f>
-        <v>130583</v>
+        <v>12380</v>
       </c>
       <c r="G964" s="42">
         <v>2461</v>
@@ -46273,7 +46273,7 @@
         <v>1429</v>
       </c>
       <c r="G1065" s="48" t="s">
-        <v>2348</v>
+        <v>2353</v>
       </c>
       <c r="H1065" s="20" t="s">
         <v>1631</v>
@@ -46309,7 +46309,7 @@
         <v>3591</v>
       </c>
       <c r="G1066" s="48" t="s">
-        <v>2348</v>
+        <v>2353</v>
       </c>
       <c r="H1066" s="20" t="s">
         <v>1631</v>
@@ -46345,7 +46345,7 @@
         <v>24746</v>
       </c>
       <c r="G1067" s="48" t="s">
-        <v>2348</v>
+        <v>2353</v>
       </c>
       <c r="H1067" s="20" t="s">
         <v>1631</v>
@@ -46381,7 +46381,7 @@
         <v>856</v>
       </c>
       <c r="G1068" s="48" t="s">
-        <v>2348</v>
+        <v>2353</v>
       </c>
       <c r="H1068" s="20" t="s">
         <v>1631</v>
@@ -47603,7 +47603,7 @@
         <v>152775</v>
       </c>
       <c r="G1102" s="42" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="H1102" s="11">
         <v>46117</v>
@@ -47639,7 +47639,7 @@
         <v>43125</v>
       </c>
       <c r="G1103" s="42" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="H1103" s="11">
         <v>46117</v>
@@ -47675,7 +47675,7 @@
         <v>3300</v>
       </c>
       <c r="G1104" s="42" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="H1104" s="11">
         <v>46117</v>
@@ -47711,7 +47711,7 @@
         <v>580</v>
       </c>
       <c r="G1105" s="42" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="H1105" s="11">
         <v>46117</v>
@@ -47747,7 +47747,7 @@
         <v>220</v>
       </c>
       <c r="G1106" s="42" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="H1106" s="11">
         <v>46117</v>
@@ -64603,7 +64603,7 @@
     <row r="1576" spans="1:11" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="F1576" s="67">
         <f>SUM(F2:F1575)</f>
-        <v>26124894.386196017</v>
+        <v>26006691.386196017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update all.xlsx with additional transaction data
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56A6023-71DF-4007-9AE5-C1A077E83A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1404FAAB-8975-4C67-B2DE-EBA265FA7649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31455,7 +31455,7 @@
         <v>1990</v>
       </c>
       <c r="G653" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H653" s="11" t="s">
         <v>1148</v>
@@ -31491,7 +31491,7 @@
         <v>789.75</v>
       </c>
       <c r="G654" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H654" s="11" t="s">
         <v>1148</v>
@@ -31527,7 +31527,7 @@
         <v>526.5</v>
       </c>
       <c r="G655" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H655" s="11" t="s">
         <v>1148</v>
@@ -31563,7 +31563,7 @@
         <v>6142.5</v>
       </c>
       <c r="G656" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H656" s="11" t="s">
         <v>1148</v>
@@ -31599,7 +31599,7 @@
         <v>99.54</v>
       </c>
       <c r="G657" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H657" s="11" t="s">
         <v>1148</v>
@@ -31635,7 +31635,7 @@
         <v>10750.320000000002</v>
       </c>
       <c r="G658" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H658" s="11" t="s">
         <v>1148</v>
@@ -31671,7 +31671,7 @@
         <v>2340</v>
       </c>
       <c r="G659" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H659" s="11" t="s">
         <v>1148</v>
@@ -31707,7 +31707,7 @@
         <v>351</v>
       </c>
       <c r="G660" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H660" s="11" t="s">
         <v>1148</v>
@@ -31743,7 +31743,7 @@
         <v>2290.62</v>
       </c>
       <c r="G661" s="42">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H661" s="11" t="s">
         <v>1148</v>

</xml_diff>

<commit_message>
Update all.xlsx with new transaction data
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1404FAAB-8975-4C67-B2DE-EBA265FA7649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D9812B-44E9-4859-BC35-C3C75FDF4D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8400" uniqueCount="2354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8408" uniqueCount="2355">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7099,6 +7099,9 @@
   </si>
   <si>
     <t>RAW/M/2026/0001755</t>
+  </si>
+  <si>
+    <t>HQ89598</t>
   </si>
 </sst>
 </file>
@@ -7957,7 +7960,7 @@
     <col min="6" max="6" width="19.7109375" style="66" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="28.28515625" style="49" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" style="60" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.42578125" style="49" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.5703125" style="49" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.28515625" style="49" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" style="60" bestFit="1" customWidth="1"/>
   </cols>
@@ -31814,14 +31817,14 @@
         <f t="shared" si="10"/>
         <v>3215</v>
       </c>
-      <c r="G663" s="42">
-        <v>89598</v>
+      <c r="G663" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H663" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I663" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J663" s="42">
         <v>6250</v>
@@ -31850,14 +31853,14 @@
         <f t="shared" si="10"/>
         <v>346</v>
       </c>
-      <c r="G664" s="42">
-        <v>89598</v>
+      <c r="G664" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H664" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I664" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J664" s="42">
         <v>6250</v>
@@ -31886,14 +31889,14 @@
         <f t="shared" si="10"/>
         <v>354</v>
       </c>
-      <c r="G665" s="42">
-        <v>89598</v>
+      <c r="G665" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H665" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I665" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J665" s="42">
         <v>6250</v>
@@ -31922,14 +31925,14 @@
         <f t="shared" si="10"/>
         <v>1218</v>
       </c>
-      <c r="G666" s="42">
-        <v>89598</v>
+      <c r="G666" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H666" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I666" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J666" s="42">
         <v>6250</v>
@@ -31958,14 +31961,14 @@
         <f t="shared" si="10"/>
         <v>346</v>
       </c>
-      <c r="G667" s="42">
-        <v>89598</v>
+      <c r="G667" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H667" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I667" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J667" s="42">
         <v>6250</v>
@@ -31994,14 +31997,14 @@
         <f t="shared" si="10"/>
         <v>1105</v>
       </c>
-      <c r="G668" s="42">
-        <v>89598</v>
+      <c r="G668" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H668" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I668" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J668" s="42">
         <v>6250</v>
@@ -32030,14 +32033,14 @@
         <f t="shared" si="10"/>
         <v>1057</v>
       </c>
-      <c r="G669" s="42">
-        <v>89598</v>
+      <c r="G669" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H669" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I669" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J669" s="42">
         <v>6250</v>
@@ -32066,14 +32069,14 @@
         <f t="shared" si="10"/>
         <v>362</v>
       </c>
-      <c r="G670" s="42">
-        <v>89598</v>
+      <c r="G670" s="42" t="s">
+        <v>2354</v>
       </c>
       <c r="H670" s="11" t="s">
         <v>1164</v>
       </c>
       <c r="I670" s="42" t="s">
-        <v>116</v>
+        <v>607</v>
       </c>
       <c r="J670" s="42">
         <v>6250</v>

</xml_diff>